<commit_message>
Refresh final dissertation outputs
</commit_message>
<xml_diff>
--- a/4_outputs/final/Table05.xlsx
+++ b/4_outputs/final/Table05.xlsx
@@ -421,7 +421,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
@@ -430,12 +430,12 @@
       <c r="A1" s="1" t="inlineStr"/>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Semantic Gap</t>
+          <t>Raw Gap</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Adj. gap</t>
+          <t>Adj. Gap</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">

</xml_diff>